<commit_message>
[New] Se agregan funcionalidades asociadas al chat con IA
</commit_message>
<xml_diff>
--- a/uploads/extensiones_teams_1.xlsx
+++ b/uploads/extensiones_teams_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mafred\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC061C7-A5FF-4FBA-BDD6-F9CA1E188949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0D9FC6-CC89-4DD9-B424-9F7AA72106FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2620" yWindow="2620" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="alta o baja" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>correo</t>
   </si>
@@ -44,38 +44,20 @@
     <t>código de país + número_alta</t>
   </si>
   <si>
-    <t>Manfred@gmail.com</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>50661615217</t>
-  </si>
-  <si>
-    <t>Manfred1@gmail.com</t>
-  </si>
-  <si>
-    <t>Manfred2@gmail.com</t>
-  </si>
-  <si>
-    <t>Manfred3@gmail.com</t>
-  </si>
-  <si>
-    <t>Manfred4@gmail.com</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>50640004000</t>
+    <t>masuarezb@grupobisa.com</t>
+  </si>
+  <si>
+    <t>fvela@grupobisa.com</t>
+  </si>
+  <si>
+    <t>59122317272</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,14 +69,6 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -147,21 +121,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -465,18 +436,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1"/>
-    <col min="5" max="5" width="39.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="30.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.81640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" style="1"/>
+    <col min="5" max="5" width="39.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -487,42 +458,54 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
+      <c r="B2" s="1">
+        <v>2218</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1139</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E8" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{AE3DFD9F-73A1-45C1-B7C3-A94B928DEF64}"/>
+    <hyperlink ref="A2" r:id="rId1" display="mailto:masuarezb@grupobisa.com" xr:uid="{E3A0B686-F0FF-4345-9B2E-6B10EA24DEF7}"/>
+    <hyperlink ref="A3" r:id="rId2" display="mailto:fvela@grupobisa.com" xr:uid="{E5B413D5-C50E-4BA6-82C9-23D9139B7820}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FE848B-5110-40D5-8B94-A2348EA5BBB0}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7265625" style="1" customWidth="1"/>
     <col min="3" max="3" width="30" style="1" customWidth="1"/>
     <col min="4" max="4" width="29" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.7109375" customWidth="1"/>
+    <col min="5" max="6" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -536,41 +519,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{1FC1D324-B990-4BE3-BBF9-C4D07895057D}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{8A6C7B32-2802-4A31-9645-E1B2F281D930}"/>
-    <hyperlink ref="D2" r:id="rId3" xr:uid="{C5D6F553-B722-42F6-8AAC-9BD21E960DF9}"/>
-    <hyperlink ref="D3" r:id="rId4" xr:uid="{EE5686F4-3441-4564-A0E1-DFBF9D414ECF}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>